<commit_message>
fix bugs on tests
</commit_message>
<xml_diff>
--- a/Banlic-Mamatid_traci/batch_results/DDPG_Results.xlsx
+++ b/Banlic-Mamatid_traci/batch_results/DDPG_Results.xlsx
@@ -627,16 +627,16 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>68.1099</v>
+        <v>80.09950000000001</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>118.9862</v>
+        <v>114.5868</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>9.7232</v>
+        <v>12.1507</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>2695.1625</v>
+        <v>2642.6813</v>
       </c>
     </row>
     <row r="6" ht="14" customHeight="1">
@@ -646,16 +646,16 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>68.7739</v>
+        <v>77.2916</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>111.2709</v>
+        <v>113.0365</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>10.4602</v>
+        <v>11.886</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>2651.5554</v>
+        <v>2730.3939</v>
       </c>
     </row>
     <row r="7" ht="14" customHeight="1">
@@ -665,16 +665,16 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>71.1678</v>
+        <v>78.3308</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>109.9898</v>
+        <v>110.6656</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>10.1764</v>
+        <v>11.5508</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>2715.9027</v>
+        <v>2759.1308</v>
       </c>
     </row>
     <row r="8" ht="14" customHeight="1">
@@ -684,16 +684,16 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>69.289</v>
+        <v>80.6478</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>116.2532</v>
+        <v>118.079</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>9.7104</v>
+        <v>11.8071</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>2654.1061</v>
+        <v>2634.0782</v>
       </c>
     </row>
     <row r="9" ht="14" customHeight="1">
@@ -703,16 +703,16 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>68.3159</v>
+        <v>80.3411</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>112.6256</v>
+        <v>118.91</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>9.8072</v>
+        <v>11.3794</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>2552.3008</v>
+        <v>2490.5189</v>
       </c>
     </row>
     <row r="10" ht="14" customHeight="1">
@@ -722,16 +722,16 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>70.1515</v>
+        <v>80.8158</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>110.9349</v>
+        <v>115.1487</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>11.4766</v>
+        <v>13.9572</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>2832.2753</v>
+        <v>2770.1576</v>
       </c>
     </row>
     <row r="11" ht="14" customHeight="1">
@@ -741,16 +741,16 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>69.66679999999999</v>
+        <v>82.2132</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>118.0509</v>
+        <v>118.1661</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>10.4897</v>
+        <v>12.4361</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>2719.221</v>
+        <v>2735.0021</v>
       </c>
     </row>
     <row r="12" ht="14" customHeight="1">
@@ -760,16 +760,16 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>72.1746</v>
+        <v>82.64100000000001</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>116.0841</v>
+        <v>118.001</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>10.8876</v>
+        <v>13.3406</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>2740.9994</v>
+        <v>2711.1996</v>
       </c>
     </row>
     <row r="13" ht="14" customHeight="1">
@@ -779,16 +779,16 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>70.035</v>
+        <v>80.9503</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>106.5876</v>
+        <v>111.3131</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>10.7296</v>
+        <v>12.8954</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>2754.6028</v>
+        <v>2754.9449</v>
       </c>
     </row>
     <row r="14" ht="14" customHeight="1">
@@ -798,16 +798,16 @@
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>70.6138</v>
+        <v>76.4629</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>114.7528</v>
+        <v>119.9482</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>10.0722</v>
+        <v>11.3319</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>2692.3983</v>
+        <v>2754.9178</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
@@ -824,16 +824,16 @@
         </is>
       </c>
       <c r="B16" s="9" t="n">
-        <v>179.8554</v>
+        <v>280.4123</v>
       </c>
       <c r="C16" s="9" t="n">
-        <v>136.1956</v>
+        <v>126.7063</v>
       </c>
       <c r="D16" s="9" t="n">
-        <v>36.9333</v>
+        <v>35.256</v>
       </c>
       <c r="E16" s="9" t="n">
-        <v>6045.561</v>
+        <v>5140.7346</v>
       </c>
     </row>
     <row r="17" ht="14" customHeight="1">
@@ -843,16 +843,16 @@
         </is>
       </c>
       <c r="B17" s="9" t="n">
-        <v>109.8539</v>
+        <v>186.277</v>
       </c>
       <c r="C17" s="9" t="n">
-        <v>129.0713</v>
+        <v>132.9486</v>
       </c>
       <c r="D17" s="9" t="n">
-        <v>30.1823</v>
+        <v>38.4445</v>
       </c>
       <c r="E17" s="9" t="n">
-        <v>5616.523</v>
+        <v>5459.3642</v>
       </c>
     </row>
     <row r="18" ht="14" customHeight="1">
@@ -862,16 +862,16 @@
         </is>
       </c>
       <c r="B18" s="9" t="n">
-        <v>128.5555</v>
+        <v>188.4106</v>
       </c>
       <c r="C18" s="9" t="n">
-        <v>136.6993</v>
+        <v>125.5958</v>
       </c>
       <c r="D18" s="9" t="n">
-        <v>34.6261</v>
+        <v>35.8811</v>
       </c>
       <c r="E18" s="9" t="n">
-        <v>5711.0558</v>
+        <v>5370.723</v>
       </c>
     </row>
     <row r="19" ht="14" customHeight="1">
@@ -881,16 +881,16 @@
         </is>
       </c>
       <c r="B19" s="9" t="n">
-        <v>101.5887</v>
+        <v>163.6761</v>
       </c>
       <c r="C19" s="9" t="n">
-        <v>125.3454</v>
+        <v>148.633</v>
       </c>
       <c r="D19" s="9" t="n">
-        <v>28.4056</v>
+        <v>35.5914</v>
       </c>
       <c r="E19" s="9" t="n">
-        <v>5554.4752</v>
+        <v>5638.4918</v>
       </c>
     </row>
     <row r="20" ht="14" customHeight="1">
@@ -900,16 +900,16 @@
         </is>
       </c>
       <c r="B20" s="9" t="n">
-        <v>110.8159</v>
+        <v>161.2474</v>
       </c>
       <c r="C20" s="9" t="n">
-        <v>121.8455</v>
+        <v>140.8408</v>
       </c>
       <c r="D20" s="9" t="n">
-        <v>30.4406</v>
+        <v>42.4158</v>
       </c>
       <c r="E20" s="9" t="n">
-        <v>5601.9161</v>
+        <v>5874.9064</v>
       </c>
     </row>
     <row r="21" ht="14" customHeight="1">
@@ -919,16 +919,16 @@
         </is>
       </c>
       <c r="B21" s="9" t="n">
-        <v>133.9924</v>
+        <v>167.1945</v>
       </c>
       <c r="C21" s="9" t="n">
-        <v>129.4708</v>
+        <v>153.1466</v>
       </c>
       <c r="D21" s="9" t="n">
-        <v>32.3656</v>
+        <v>38.0224</v>
       </c>
       <c r="E21" s="9" t="n">
-        <v>5578.0776</v>
+        <v>5606.7264</v>
       </c>
     </row>
     <row r="22" ht="14" customHeight="1">
@@ -938,16 +938,16 @@
         </is>
       </c>
       <c r="B22" s="9" t="n">
-        <v>92.5796</v>
+        <v>216.6424</v>
       </c>
       <c r="C22" s="9" t="n">
-        <v>115.6039</v>
+        <v>126.5588</v>
       </c>
       <c r="D22" s="9" t="n">
-        <v>29.3909</v>
+        <v>38.0132</v>
       </c>
       <c r="E22" s="9" t="n">
-        <v>5619.9552</v>
+        <v>5369.6948</v>
       </c>
     </row>
     <row r="23" ht="14" customHeight="1">
@@ -957,16 +957,16 @@
         </is>
       </c>
       <c r="B23" s="9" t="n">
-        <v>91.8663</v>
+        <v>184.1107</v>
       </c>
       <c r="C23" s="9" t="n">
-        <v>123.5552</v>
+        <v>126.9312</v>
       </c>
       <c r="D23" s="9" t="n">
-        <v>29.4465</v>
+        <v>37.2443</v>
       </c>
       <c r="E23" s="9" t="n">
-        <v>5814.3729</v>
+        <v>5725.512</v>
       </c>
     </row>
     <row r="24" ht="14" customHeight="1">
@@ -976,16 +976,16 @@
         </is>
       </c>
       <c r="B24" s="9" t="n">
-        <v>99.22410000000001</v>
+        <v>154.6267</v>
       </c>
       <c r="C24" s="9" t="n">
-        <v>128.5628</v>
+        <v>138.4848</v>
       </c>
       <c r="D24" s="9" t="n">
-        <v>30.3378</v>
+        <v>36.2222</v>
       </c>
       <c r="E24" s="9" t="n">
-        <v>5577.5426</v>
+        <v>5658.557</v>
       </c>
     </row>
     <row r="25" ht="14" customHeight="1">
@@ -995,16 +995,16 @@
         </is>
       </c>
       <c r="B25" s="9" t="n">
-        <v>157.4948</v>
+        <v>302.9529</v>
       </c>
       <c r="C25" s="9" t="n">
-        <v>137.9377</v>
+        <v>126.5801</v>
       </c>
       <c r="D25" s="9" t="n">
-        <v>35.4115</v>
+        <v>35.4102</v>
       </c>
       <c r="E25" s="9" t="n">
-        <v>5842.4741</v>
+        <v>5049.0033</v>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
@@ -1021,16 +1021,16 @@
         </is>
       </c>
       <c r="B27" s="12" t="n">
-        <v>578.0872000000001</v>
+        <v>677.0836</v>
       </c>
       <c r="C27" s="12" t="n">
-        <v>140.2409</v>
+        <v>138.4026</v>
       </c>
       <c r="D27" s="12" t="n">
-        <v>46.591</v>
+        <v>40.4951</v>
       </c>
       <c r="E27" s="12" t="n">
-        <v>6385.4791</v>
+        <v>5463.6036</v>
       </c>
     </row>
     <row r="28" ht="14" customHeight="1">
@@ -1040,16 +1040,16 @@
         </is>
       </c>
       <c r="B28" s="12" t="n">
-        <v>548.9811999999999</v>
+        <v>760.2928000000001</v>
       </c>
       <c r="C28" s="12" t="n">
-        <v>146.5978</v>
+        <v>145.6773</v>
       </c>
       <c r="D28" s="12" t="n">
-        <v>45.9192</v>
+        <v>39.1594</v>
       </c>
       <c r="E28" s="12" t="n">
-        <v>6622.0186</v>
+        <v>4881.6477</v>
       </c>
     </row>
     <row r="29" ht="14" customHeight="1">
@@ -1059,16 +1059,16 @@
         </is>
       </c>
       <c r="B29" s="12" t="n">
-        <v>582.9439</v>
+        <v>757.3504</v>
       </c>
       <c r="C29" s="12" t="n">
-        <v>145.1572</v>
+        <v>143.4183</v>
       </c>
       <c r="D29" s="12" t="n">
-        <v>44.7884</v>
+        <v>39.6768</v>
       </c>
       <c r="E29" s="12" t="n">
-        <v>6615.916</v>
+        <v>5188.3167</v>
       </c>
     </row>
     <row r="30" ht="14" customHeight="1">
@@ -1078,16 +1078,16 @@
         </is>
       </c>
       <c r="B30" s="12" t="n">
-        <v>587.5399</v>
+        <v>818.6692</v>
       </c>
       <c r="C30" s="12" t="n">
-        <v>128.2897</v>
+        <v>151.7456</v>
       </c>
       <c r="D30" s="12" t="n">
-        <v>40.3893</v>
+        <v>40.7819</v>
       </c>
       <c r="E30" s="12" t="n">
-        <v>6102.0125</v>
+        <v>4937.8522</v>
       </c>
     </row>
     <row r="31" ht="14" customHeight="1">
@@ -1097,16 +1097,16 @@
         </is>
       </c>
       <c r="B31" s="12" t="n">
-        <v>616.2147</v>
+        <v>1040.2728</v>
       </c>
       <c r="C31" s="12" t="n">
-        <v>147.6737</v>
+        <v>439.2398</v>
       </c>
       <c r="D31" s="12" t="n">
-        <v>48.6105</v>
+        <v>42.3482</v>
       </c>
       <c r="E31" s="12" t="n">
-        <v>6647.4369</v>
+        <v>4987.4786</v>
       </c>
     </row>
     <row r="32" ht="14" customHeight="1">
@@ -1116,16 +1116,16 @@
         </is>
       </c>
       <c r="B32" s="12" t="n">
-        <v>590.022</v>
+        <v>679.3285</v>
       </c>
       <c r="C32" s="12" t="n">
-        <v>132.5524</v>
+        <v>123.316</v>
       </c>
       <c r="D32" s="12" t="n">
-        <v>44.5325</v>
+        <v>42.8806</v>
       </c>
       <c r="E32" s="12" t="n">
-        <v>6050.4104</v>
+        <v>5613.5542</v>
       </c>
     </row>
     <row r="33" ht="14" customHeight="1">
@@ -1135,16 +1135,16 @@
         </is>
       </c>
       <c r="B33" s="12" t="n">
-        <v>610.0405</v>
+        <v>742.8680000000001</v>
       </c>
       <c r="C33" s="12" t="n">
-        <v>1107.3776</v>
+        <v>144.5015</v>
       </c>
       <c r="D33" s="12" t="n">
-        <v>29.1002</v>
+        <v>39.6071</v>
       </c>
       <c r="E33" s="12" t="n">
-        <v>3837.774</v>
+        <v>5218.6867</v>
       </c>
     </row>
     <row r="34" ht="14" customHeight="1">
@@ -1154,16 +1154,16 @@
         </is>
       </c>
       <c r="B34" s="12" t="n">
-        <v>513.5242</v>
+        <v>786.9069</v>
       </c>
       <c r="C34" s="12" t="n">
-        <v>126.5667</v>
+        <v>151.0578</v>
       </c>
       <c r="D34" s="12" t="n">
-        <v>39.3674</v>
+        <v>37.0598</v>
       </c>
       <c r="E34" s="12" t="n">
-        <v>5963.7138</v>
+        <v>4912.5965</v>
       </c>
     </row>
     <row r="35" ht="14" customHeight="1">
@@ -1173,16 +1173,16 @@
         </is>
       </c>
       <c r="B35" s="12" t="n">
-        <v>547.4767000000001</v>
+        <v>740.7773999999999</v>
       </c>
       <c r="C35" s="12" t="n">
-        <v>154.2922</v>
+        <v>161.0028</v>
       </c>
       <c r="D35" s="12" t="n">
-        <v>48.1367</v>
+        <v>43.6652</v>
       </c>
       <c r="E35" s="12" t="n">
-        <v>6456.8183</v>
+        <v>5747.1231</v>
       </c>
     </row>
     <row r="36" ht="14" customHeight="1">
@@ -1192,16 +1192,16 @@
         </is>
       </c>
       <c r="B36" s="12" t="n">
-        <v>641.2744</v>
+        <v>941.487</v>
       </c>
       <c r="C36" s="12" t="n">
-        <v>147.6029</v>
+        <v>159.9488</v>
       </c>
       <c r="D36" s="12" t="n">
-        <v>48.95</v>
+        <v>43.3864</v>
       </c>
       <c r="E36" s="12" t="n">
-        <v>6446.3222</v>
+        <v>5186.271</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">

</xml_diff>